<commit_message>
add and reorg files
</commit_message>
<xml_diff>
--- a/Calibrations/CalibrationsSummary_2026-06-02-AJE.xlsx
+++ b/Calibrations/CalibrationsSummary_2026-06-02-AJE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milli079\Documents\GitHub\SAFL-Mesocosms\Calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E41BCC6-6764-4EC4-9B78-D1F1F463C8DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BDDDEA1-A1D5-46AE-B79E-8F55DBF13B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{97F5D55E-0765-4069-8CF4-3533445EA4CE}"/>
+    <workbookView xWindow="-24120" yWindow="660" windowWidth="24240" windowHeight="13020" xr2:uid="{97F5D55E-0765-4069-8CF4-3533445EA4CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -555,7 +555,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -632,6 +632,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1978,7 +1979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3576EF09-CAB0-463D-AB3F-0D14EA8E7E8F}">
-  <dimension ref="B1:P25"/>
+  <dimension ref="B1:P27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
@@ -3197,6 +3198,16 @@
       <c r="P25" s="25" t="e">
         <f t="shared" si="8"/>
         <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="H27" s="38">
+        <f>AVERAGE(H8:H23)</f>
+        <v>1.2791592416916934E-2</v>
+      </c>
+      <c r="P27" s="38">
+        <f>AVERAGE(P9:P23)</f>
+        <v>3.4681592096270373E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final commit of intial testing
</commit_message>
<xml_diff>
--- a/Calibrations/CalibrationsSummary_2026-06-02-AJE.xlsx
+++ b/Calibrations/CalibrationsSummary_2026-06-02-AJE.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\milli079\Documents\GitHub\SAFL-Mesocosms\Calibrations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BDDDEA1-A1D5-46AE-B79E-8F55DBF13B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEBEB5B6-8019-4141-A76F-7509F3D599CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="660" windowWidth="24240" windowHeight="13020" xr2:uid="{97F5D55E-0765-4069-8CF4-3533445EA4CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97F5D55E-0765-4069-8CF4-3533445EA4CE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="2026-06-02" sheetId="1" r:id="rId1"/>
+    <sheet name="2026-06-08" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,8 +39,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="21">
   <si>
     <t>Test Weight</t>
   </si>
@@ -67,6 +90,62 @@
   <si>
     <t>(percent)</t>
   </si>
+  <si>
+    <t>mV</t>
+  </si>
+  <si>
+    <t>mV zeroed</t>
+  </si>
+  <si>
+    <t>Slope</t>
+  </si>
+  <si>
+    <t>Offset</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Avg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equation (using LINEST) </t>
+  </si>
+  <si>
+    <t>TEST DATA FROM JUNE 8, 2026</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Note:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  I forced the intercept to be 0.  I think this is the right idea, but maybe I'm just skewing the data? </t>
+    </r>
+  </si>
+  <si>
+    <t>DATA FROM JUNE 1, 2026 (Used for Equation)</t>
+  </si>
 </sst>
 </file>
 
@@ -76,7 +155,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,16 +186,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="33">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -550,12 +643,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -596,6 +715,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -632,7 +752,58 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1996,79 +2167,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="29"/>
       <c r="H1" s="21"/>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
-      <c r="O1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="29"/>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="29"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="31"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="32"/>
       <c r="H2" s="22"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="31"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="32"/>
     </row>
     <row r="3" spans="2:16" ht="278.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="32"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="34"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="35"/>
       <c r="H3" s="22"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="34"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="34"/>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="35"/>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B4" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="35" t="s">
+      <c r="B4" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="37"/>
+      <c r="D4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="36"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="37"/>
       <c r="G4" s="13" t="s">
         <v>7</v>
       </c>
       <c r="H4" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="35" t="s">
-        <v>0</v>
-      </c>
-      <c r="K4" s="36"/>
-      <c r="L4" s="35" t="s">
+      <c r="J4" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" s="37"/>
+      <c r="L4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="M4" s="37"/>
-      <c r="N4" s="36"/>
+      <c r="M4" s="38"/>
+      <c r="N4" s="37"/>
       <c r="O4" s="13" t="s">
         <v>7</v>
       </c>
@@ -2548,7 +2719,7 @@
         <v>53.977492029998757</v>
       </c>
       <c r="P13" s="25">
-        <f t="shared" si="8"/>
+        <f>O13/K13</f>
         <v>3.4313725490195284E-3</v>
       </c>
     </row>
@@ -3201,11 +3372,11 @@
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="H27" s="38">
+      <c r="H27" s="26">
         <f>AVERAGE(H8:H23)</f>
         <v>1.2791592416916934E-2</v>
       </c>
-      <c r="P27" s="38">
+      <c r="P27" s="26">
         <f>AVERAGE(P9:P23)</f>
         <v>3.4681592096270373E-3</v>
       </c>
@@ -3264,4 +3435,1005 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AB18ED5-2A8B-4789-9693-76BD26AAA1D4}">
+  <dimension ref="B3:P27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="13" max="13" width="11.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="67"/>
+      <c r="D3" s="67"/>
+      <c r="E3" s="67"/>
+      <c r="J3" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="67"/>
+      <c r="L3" s="67"/>
+      <c r="M3" s="67"/>
+      <c r="N3" s="67"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="67"/>
+    </row>
+    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B4" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="43"/>
+      <c r="D4" s="42" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="43"/>
+      <c r="G4" s="63" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="64"/>
+      <c r="J4" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" s="37"/>
+      <c r="L4" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="38"/>
+      <c r="N4" s="37"/>
+      <c r="O4" s="42" t="s">
+        <v>7</v>
+      </c>
+      <c r="P4" s="43"/>
+    </row>
+    <row r="5" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="59" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="60" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="65" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="66" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="N5" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="P5" s="41" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="55">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4">
+        <f>B6*453.59237</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="55">
+        <v>0.05</v>
+      </c>
+      <c r="E6" s="56">
+        <f>D6-$D$6</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="61" cm="1">
+        <f t="array" ref="G6:H6">LINEST(C6:C25,E6:E25,FALSE,FALSE)</f>
+        <v>1506.3586029839364</v>
+      </c>
+      <c r="H6" s="62">
+        <v>0</v>
+      </c>
+      <c r="J6" s="55">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4">
+        <f>J6*453.59237</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="55">
+        <v>0.06</v>
+      </c>
+      <c r="M6" s="44">
+        <f>L6-$L$6</f>
+        <v>0</v>
+      </c>
+      <c r="N6" s="56">
+        <f>M6*G$6+$H$6</f>
+        <v>0</v>
+      </c>
+      <c r="O6" s="57">
+        <f>ABS(N6-K6)</f>
+        <v>0</v>
+      </c>
+      <c r="P6" s="58">
+        <f>IF(O6=0,0,O6/K6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B7" s="46">
+        <v>0</v>
+      </c>
+      <c r="C7" s="6">
+        <f t="shared" ref="C7:C25" si="0">B7*453.59237</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="46">
+        <v>0.05</v>
+      </c>
+      <c r="E7" s="48">
+        <f>D7-$D$6</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="31"/>
+      <c r="J7" s="46">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <f t="shared" ref="K7:K24" si="1">J7*453.59237</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="46">
+        <v>0.06</v>
+      </c>
+      <c r="M7" s="45">
+        <f>L7-$L$6</f>
+        <v>0</v>
+      </c>
+      <c r="N7" s="56">
+        <f t="shared" ref="N7:N24" si="2">M7*G$6+$H$6</f>
+        <v>0</v>
+      </c>
+      <c r="O7" s="51">
+        <f t="shared" ref="O7:O24" si="3">ABS(N7-K7)</f>
+        <v>0</v>
+      </c>
+      <c r="P7" s="52">
+        <f t="shared" ref="P7:P24" si="4">IF(O7=0,0,O7/K7)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B8" s="46">
+        <v>1.77</v>
+      </c>
+      <c r="C8" s="6">
+        <f t="shared" si="0"/>
+        <v>802.85849489999998</v>
+      </c>
+      <c r="D8" s="46">
+        <v>0.59</v>
+      </c>
+      <c r="E8" s="48">
+        <f>D8-$D$6</f>
+        <v>0.53999999999999992</v>
+      </c>
+      <c r="G8" s="68"/>
+      <c r="H8" s="68"/>
+      <c r="J8" s="46">
+        <v>1.8</v>
+      </c>
+      <c r="K8" s="6">
+        <f t="shared" si="1"/>
+        <v>816.46626600000002</v>
+      </c>
+      <c r="L8" s="46">
+        <v>0.6</v>
+      </c>
+      <c r="M8" s="45">
+        <f>L8-$L$6</f>
+        <v>0.54</v>
+      </c>
+      <c r="N8" s="56">
+        <f t="shared" si="2"/>
+        <v>813.43364561132569</v>
+      </c>
+      <c r="O8" s="51">
+        <f t="shared" si="3"/>
+        <v>3.0326203886743315</v>
+      </c>
+      <c r="P8" s="52">
+        <f t="shared" si="4"/>
+        <v>3.7143241735284765E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B9" s="46">
+        <v>5.17</v>
+      </c>
+      <c r="C9" s="6">
+        <f t="shared" si="0"/>
+        <v>2345.0725529000001</v>
+      </c>
+      <c r="D9" s="46">
+        <v>1.6</v>
+      </c>
+      <c r="E9" s="48">
+        <f>D9-$D$6</f>
+        <v>1.55</v>
+      </c>
+      <c r="G9" s="68"/>
+      <c r="H9" s="68"/>
+      <c r="J9" s="46">
+        <v>5.76</v>
+      </c>
+      <c r="K9" s="6">
+        <f t="shared" si="1"/>
+        <v>2612.6920512000002</v>
+      </c>
+      <c r="L9" s="46">
+        <v>1.8</v>
+      </c>
+      <c r="M9" s="45">
+        <f>L9-$L$6</f>
+        <v>1.74</v>
+      </c>
+      <c r="N9" s="56">
+        <f t="shared" si="2"/>
+        <v>2621.0639691920492</v>
+      </c>
+      <c r="O9" s="51">
+        <f t="shared" si="3"/>
+        <v>8.3719179920490205</v>
+      </c>
+      <c r="P9" s="52">
+        <f t="shared" si="4"/>
+        <v>3.2043263530441056E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B10" s="46">
+        <v>11.25</v>
+      </c>
+      <c r="C10" s="6">
+        <f t="shared" si="0"/>
+        <v>5102.9141625000002</v>
+      </c>
+      <c r="D10" s="46">
+        <v>3.44</v>
+      </c>
+      <c r="E10" s="48">
+        <f>D10-$D$6</f>
+        <v>3.39</v>
+      </c>
+      <c r="G10" s="68"/>
+      <c r="H10" s="68"/>
+      <c r="J10" s="46">
+        <v>10.78</v>
+      </c>
+      <c r="K10" s="6">
+        <f t="shared" si="1"/>
+        <v>4889.7257485999999</v>
+      </c>
+      <c r="L10" s="46">
+        <v>3.3</v>
+      </c>
+      <c r="M10" s="45">
+        <f>L10-$L$6</f>
+        <v>3.2399999999999998</v>
+      </c>
+      <c r="N10" s="56">
+        <f t="shared" si="2"/>
+        <v>4880.6018736679534</v>
+      </c>
+      <c r="O10" s="51">
+        <f t="shared" si="3"/>
+        <v>9.1238749320464194</v>
+      </c>
+      <c r="P10" s="52">
+        <f t="shared" si="4"/>
+        <v>1.865927743423794E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B11" s="46">
+        <v>18.96</v>
+      </c>
+      <c r="C11" s="6">
+        <f t="shared" si="0"/>
+        <v>8600.1113352000011</v>
+      </c>
+      <c r="D11" s="46">
+        <v>5.76</v>
+      </c>
+      <c r="E11" s="48">
+        <f>D11-$D$6</f>
+        <v>5.71</v>
+      </c>
+      <c r="G11" s="68"/>
+      <c r="H11" s="68"/>
+      <c r="J11" s="46">
+        <v>16.84</v>
+      </c>
+      <c r="K11" s="6">
+        <f t="shared" si="1"/>
+        <v>7638.4955108000004</v>
+      </c>
+      <c r="L11" s="46">
+        <v>5.13</v>
+      </c>
+      <c r="M11" s="45">
+        <f>L11-$L$6</f>
+        <v>5.07</v>
+      </c>
+      <c r="N11" s="56">
+        <f t="shared" si="2"/>
+        <v>7637.2381171285579</v>
+      </c>
+      <c r="O11" s="51">
+        <f t="shared" si="3"/>
+        <v>1.2573936714425145</v>
+      </c>
+      <c r="P11" s="52">
+        <f t="shared" si="4"/>
+        <v>1.646127394674379E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B12" s="46">
+        <v>27.45</v>
+      </c>
+      <c r="C12" s="6">
+        <f t="shared" si="0"/>
+        <v>12451.1105565</v>
+      </c>
+      <c r="D12" s="46">
+        <v>8.31</v>
+      </c>
+      <c r="E12" s="48">
+        <f>D12-$D$6</f>
+        <v>8.26</v>
+      </c>
+      <c r="J12" s="46">
+        <v>23.66</v>
+      </c>
+      <c r="K12" s="6">
+        <f t="shared" si="1"/>
+        <v>10731.995474200001</v>
+      </c>
+      <c r="L12" s="46">
+        <v>7.18</v>
+      </c>
+      <c r="M12" s="45">
+        <f>L12-$L$6</f>
+        <v>7.12</v>
+      </c>
+      <c r="N12" s="56">
+        <f t="shared" si="2"/>
+        <v>10725.273253245627</v>
+      </c>
+      <c r="O12" s="51">
+        <f t="shared" si="3"/>
+        <v>6.7222209543742792</v>
+      </c>
+      <c r="P12" s="52">
+        <f t="shared" si="4"/>
+        <v>6.2637195203209641E-4</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B13" s="46">
+        <v>34.82</v>
+      </c>
+      <c r="C13" s="6">
+        <f t="shared" si="0"/>
+        <v>15794.086323400001</v>
+      </c>
+      <c r="D13" s="46">
+        <v>10.53</v>
+      </c>
+      <c r="E13" s="48">
+        <f>D13-$D$6</f>
+        <v>10.479999999999999</v>
+      </c>
+      <c r="J13" s="46">
+        <v>36.89</v>
+      </c>
+      <c r="K13" s="6">
+        <f t="shared" si="1"/>
+        <v>16733.0225293</v>
+      </c>
+      <c r="L13" s="46">
+        <v>11.16</v>
+      </c>
+      <c r="M13" s="45">
+        <f>L13-$L$6</f>
+        <v>11.1</v>
+      </c>
+      <c r="N13" s="56">
+        <f t="shared" si="2"/>
+        <v>16720.580493121695</v>
+      </c>
+      <c r="O13" s="51">
+        <f t="shared" si="3"/>
+        <v>12.442036178304988</v>
+      </c>
+      <c r="P13" s="52">
+        <f t="shared" si="4"/>
+        <v>7.4356178965985541E-4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B14" s="46">
+        <v>39.979999999999997</v>
+      </c>
+      <c r="C14" s="6">
+        <f t="shared" si="0"/>
+        <v>18134.622952599999</v>
+      </c>
+      <c r="D14" s="46">
+        <v>12.09</v>
+      </c>
+      <c r="E14" s="48">
+        <f>D14-$D$6</f>
+        <v>12.04</v>
+      </c>
+      <c r="J14" s="46">
+        <v>43.85</v>
+      </c>
+      <c r="K14" s="6">
+        <f t="shared" si="1"/>
+        <v>19890.0254245</v>
+      </c>
+      <c r="L14" s="46">
+        <v>13.25</v>
+      </c>
+      <c r="M14" s="45">
+        <f>L14-$L$6</f>
+        <v>13.19</v>
+      </c>
+      <c r="N14" s="56">
+        <f t="shared" si="2"/>
+        <v>19868.86997335812</v>
+      </c>
+      <c r="O14" s="51">
+        <f t="shared" si="3"/>
+        <v>21.155451141879894</v>
+      </c>
+      <c r="P14" s="52">
+        <f t="shared" si="4"/>
+        <v>1.0636211211586073E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B15" s="46">
+        <v>44.97</v>
+      </c>
+      <c r="C15" s="6">
+        <f t="shared" si="0"/>
+        <v>20398.048878900001</v>
+      </c>
+      <c r="D15" s="46">
+        <v>13.58</v>
+      </c>
+      <c r="E15" s="48">
+        <f>D15-$D$6</f>
+        <v>13.53</v>
+      </c>
+      <c r="J15" s="46">
+        <v>48.11</v>
+      </c>
+      <c r="K15" s="6">
+        <f t="shared" si="1"/>
+        <v>21822.328920700002</v>
+      </c>
+      <c r="L15" s="46">
+        <v>14.54</v>
+      </c>
+      <c r="M15" s="45">
+        <f>L15-$L$6</f>
+        <v>14.479999999999999</v>
+      </c>
+      <c r="N15" s="56">
+        <f t="shared" si="2"/>
+        <v>21812.072571207398</v>
+      </c>
+      <c r="O15" s="51">
+        <f t="shared" si="3"/>
+        <v>10.256349492603476</v>
+      </c>
+      <c r="P15" s="52">
+        <f t="shared" si="4"/>
+        <v>4.6999335084142247E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B16" s="46">
+        <v>48.07</v>
+      </c>
+      <c r="C16" s="6">
+        <f t="shared" si="0"/>
+        <v>21804.185225900001</v>
+      </c>
+      <c r="D16" s="46">
+        <v>14.53</v>
+      </c>
+      <c r="E16" s="48">
+        <f>D16-$D$6</f>
+        <v>14.479999999999999</v>
+      </c>
+      <c r="J16" s="46">
+        <v>40.81</v>
+      </c>
+      <c r="K16" s="6">
+        <f t="shared" si="1"/>
+        <v>18511.104619700003</v>
+      </c>
+      <c r="L16" s="46">
+        <v>12.33</v>
+      </c>
+      <c r="M16" s="45">
+        <f>L16-$L$6</f>
+        <v>12.27</v>
+      </c>
+      <c r="N16" s="56">
+        <f t="shared" si="2"/>
+        <v>18483.020058612899</v>
+      </c>
+      <c r="O16" s="51">
+        <f t="shared" si="3"/>
+        <v>28.084561087103793</v>
+      </c>
+      <c r="P16" s="52">
+        <f t="shared" si="4"/>
+        <v>1.5171737000079114E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B17" s="46">
+        <v>48.07</v>
+      </c>
+      <c r="C17" s="6">
+        <f t="shared" si="0"/>
+        <v>21804.185225900001</v>
+      </c>
+      <c r="D17" s="46">
+        <v>14.53</v>
+      </c>
+      <c r="E17" s="48">
+        <f>D17-$D$6</f>
+        <v>14.479999999999999</v>
+      </c>
+      <c r="J17" s="46">
+        <v>31.86</v>
+      </c>
+      <c r="K17" s="6">
+        <f t="shared" si="1"/>
+        <v>14451.452908200001</v>
+      </c>
+      <c r="L17" s="46">
+        <v>9.65</v>
+      </c>
+      <c r="M17" s="45">
+        <f>L17-$L$6</f>
+        <v>9.59</v>
+      </c>
+      <c r="N17" s="56">
+        <f t="shared" si="2"/>
+        <v>14445.97900261595</v>
+      </c>
+      <c r="O17" s="51">
+        <f t="shared" si="3"/>
+        <v>5.4739055840509536</v>
+      </c>
+      <c r="P17" s="52">
+        <f t="shared" si="4"/>
+        <v>3.7877891024680059E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B18" s="46">
+        <v>36.159999999999997</v>
+      </c>
+      <c r="C18" s="6">
+        <f t="shared" si="0"/>
+        <v>16401.9000992</v>
+      </c>
+      <c r="D18" s="46">
+        <v>10.93</v>
+      </c>
+      <c r="E18" s="48">
+        <f>D18-$D$6</f>
+        <v>10.879999999999999</v>
+      </c>
+      <c r="J18" s="46">
+        <v>20.079999999999998</v>
+      </c>
+      <c r="K18" s="6">
+        <f t="shared" si="1"/>
+        <v>9108.1347895999988</v>
+      </c>
+      <c r="L18" s="46">
+        <v>6.1</v>
+      </c>
+      <c r="M18" s="45">
+        <f>L18-$L$6</f>
+        <v>6.04</v>
+      </c>
+      <c r="N18" s="56">
+        <f t="shared" si="2"/>
+        <v>9098.4059620229764</v>
+      </c>
+      <c r="O18" s="51">
+        <f t="shared" si="3"/>
+        <v>9.7288275770224573</v>
+      </c>
+      <c r="P18" s="52">
+        <f t="shared" si="4"/>
+        <v>1.0681470796996976E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="46">
+        <v>27.5</v>
+      </c>
+      <c r="C19" s="6">
+        <f t="shared" si="0"/>
+        <v>12473.790175</v>
+      </c>
+      <c r="D19" s="46">
+        <v>8.33</v>
+      </c>
+      <c r="E19" s="48">
+        <f>D19-$D$6</f>
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="J19" s="46">
+        <v>13.26</v>
+      </c>
+      <c r="K19" s="6">
+        <f t="shared" si="1"/>
+        <v>6014.6348262000001</v>
+      </c>
+      <c r="L19" s="46">
+        <v>4.05</v>
+      </c>
+      <c r="M19" s="45">
+        <f>L19-$L$6</f>
+        <v>3.9899999999999998</v>
+      </c>
+      <c r="N19" s="56">
+        <f t="shared" si="2"/>
+        <v>6010.3708259059058</v>
+      </c>
+      <c r="O19" s="51">
+        <f t="shared" si="3"/>
+        <v>4.2640002940943305</v>
+      </c>
+      <c r="P19" s="52">
+        <f t="shared" si="4"/>
+        <v>7.0893751945174917E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B20" s="46">
+        <v>18.62</v>
+      </c>
+      <c r="C20" s="6">
+        <f t="shared" si="0"/>
+        <v>8445.8899294000003</v>
+      </c>
+      <c r="D20" s="46">
+        <v>5.68</v>
+      </c>
+      <c r="E20" s="48">
+        <f>D20-$D$6</f>
+        <v>5.63</v>
+      </c>
+      <c r="J20" s="46">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="K20" s="6">
+        <f t="shared" si="1"/>
+        <v>3764.8166710000005</v>
+      </c>
+      <c r="L20" s="46">
+        <v>2.57</v>
+      </c>
+      <c r="M20" s="45">
+        <f>L20-$L$6</f>
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="N20" s="56">
+        <f t="shared" si="2"/>
+        <v>3780.9600934896803</v>
+      </c>
+      <c r="O20" s="51">
+        <f t="shared" si="3"/>
+        <v>16.143422489679779</v>
+      </c>
+      <c r="P20" s="52">
+        <f t="shared" si="4"/>
+        <v>4.2879704114229299E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B21" s="46">
+        <v>10.87</v>
+      </c>
+      <c r="C21" s="6">
+        <f t="shared" si="0"/>
+        <v>4930.5490619000002</v>
+      </c>
+      <c r="D21" s="46">
+        <v>3.33</v>
+      </c>
+      <c r="E21" s="48">
+        <f>D21-$D$6</f>
+        <v>3.2800000000000002</v>
+      </c>
+      <c r="J21" s="46">
+        <v>5.0599999999999996</v>
+      </c>
+      <c r="K21" s="6">
+        <f t="shared" si="1"/>
+        <v>2295.1773921999998</v>
+      </c>
+      <c r="L21" s="46">
+        <v>1.58</v>
+      </c>
+      <c r="M21" s="45">
+        <f>L21-$L$6</f>
+        <v>1.52</v>
+      </c>
+      <c r="N21" s="56">
+        <f t="shared" si="2"/>
+        <v>2289.6650765355835</v>
+      </c>
+      <c r="O21" s="51">
+        <f t="shared" si="3"/>
+        <v>5.5123156644162918</v>
+      </c>
+      <c r="P21" s="52">
+        <f t="shared" si="4"/>
+        <v>2.4016948246133444E-3</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B22" s="46">
+        <v>5.05</v>
+      </c>
+      <c r="C22" s="6">
+        <f t="shared" si="0"/>
+        <v>2290.6414685</v>
+      </c>
+      <c r="D22" s="46">
+        <v>1.58</v>
+      </c>
+      <c r="E22" s="48">
+        <f>D22-$D$6</f>
+        <v>1.53</v>
+      </c>
+      <c r="J22" s="46">
+        <v>1.8</v>
+      </c>
+      <c r="K22" s="6">
+        <f t="shared" si="1"/>
+        <v>816.46626600000002</v>
+      </c>
+      <c r="L22" s="46">
+        <v>0.6</v>
+      </c>
+      <c r="M22" s="45">
+        <f>L22-$L$6</f>
+        <v>0.54</v>
+      </c>
+      <c r="N22" s="56">
+        <f t="shared" si="2"/>
+        <v>813.43364561132569</v>
+      </c>
+      <c r="O22" s="51">
+        <f t="shared" si="3"/>
+        <v>3.0326203886743315</v>
+      </c>
+      <c r="P22" s="52">
+        <f t="shared" si="4"/>
+        <v>3.7143241735284765E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B23" s="46">
+        <v>1.77</v>
+      </c>
+      <c r="C23" s="6">
+        <f t="shared" si="0"/>
+        <v>802.85849489999998</v>
+      </c>
+      <c r="D23" s="46">
+        <v>0.6</v>
+      </c>
+      <c r="E23" s="48">
+        <f>D23-$D$6</f>
+        <v>0.54999999999999993</v>
+      </c>
+      <c r="J23" s="46">
+        <v>0</v>
+      </c>
+      <c r="K23" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L23" s="46">
+        <v>0.06</v>
+      </c>
+      <c r="M23" s="45">
+        <f>L23-$L$6</f>
+        <v>0</v>
+      </c>
+      <c r="N23" s="56">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O23" s="51">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P23" s="52">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="46">
+        <v>0</v>
+      </c>
+      <c r="C24" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D24" s="46">
+        <v>0.06</v>
+      </c>
+      <c r="E24" s="48">
+        <f>D24-$D$6</f>
+        <v>9.999999999999995E-3</v>
+      </c>
+      <c r="J24" s="47">
+        <v>0</v>
+      </c>
+      <c r="K24" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L24" s="47">
+        <v>0.06</v>
+      </c>
+      <c r="M24" s="49">
+        <f>L24-$L$6</f>
+        <v>0</v>
+      </c>
+      <c r="N24" s="56">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O24" s="53">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P24" s="54">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="47">
+        <v>0</v>
+      </c>
+      <c r="C25" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D25" s="47">
+        <v>0.06</v>
+      </c>
+      <c r="E25" s="50">
+        <f>D25-$D$6</f>
+        <v>9.999999999999995E-3</v>
+      </c>
+      <c r="N25" t="s">
+        <v>14</v>
+      </c>
+      <c r="O25" s="39">
+        <f>MAX(O6:O24)</f>
+        <v>28.084561087103793</v>
+      </c>
+      <c r="P25" s="40">
+        <f>MAX(P6:P24)</f>
+        <v>4.2879704114229299E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="N26" t="s">
+        <v>15</v>
+      </c>
+      <c r="O26" s="39">
+        <f>MIN(O6:O25)</f>
+        <v>0</v>
+      </c>
+      <c r="P26" s="40">
+        <f>MIN(P6:P25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="N27" t="s">
+        <v>16</v>
+      </c>
+      <c r="O27" s="39">
+        <f>AVERAGE(O6:O26)</f>
+        <v>8.2231466154057458</v>
+      </c>
+      <c r="P27" s="40">
+        <f>AVERAGE(P6:P26)</f>
+        <v>1.4389398215976016E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="J3:P3"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="G7:H11"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="O4:O5 P5">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFFF9999"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P6:P24">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>